<commit_message>
chore: update capacity report script for April data and cleanup files
- Update file paths to point to April and May directories
- Adjust first and second week days to 25 and 24 respectively
- Extend buyer data range from G26 to G28
- Shift provision and comparison table placements down by one row
- Add .gitignore to exclude unnecessary Excel files
- Remove outdated Excel files from version control
</commit_message>
<xml_diff>
--- a/FastReact Confg..xlsx
+++ b/FastReact Confg..xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\1. Work\1. Daily\Capacity Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC51413C-8D5D-4C49-809B-204983A5B546}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19F83E07-8D07-4D4A-B6F6-9741F9826CB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="810" yWindow="-120" windowWidth="19800" windowHeight="11760" xr2:uid="{9AFED8FC-535D-48D6-A46B-931961F691BE}"/>
   </bookViews>
@@ -625,10 +625,10 @@
         <v>6</v>
       </c>
       <c r="C3" s="8">
-        <v>46082</v>
+        <v>46143</v>
       </c>
       <c r="D3" s="8">
-        <v>46234</v>
+        <v>46295</v>
       </c>
       <c r="E3" s="9" t="s">
         <v>7</v>
@@ -642,10 +642,10 @@
         <v>9</v>
       </c>
       <c r="C4" s="8">
-        <v>46054</v>
+        <v>46113</v>
       </c>
       <c r="D4" s="8">
-        <v>46234</v>
+        <v>46295</v>
       </c>
       <c r="E4" s="9" t="s">
         <v>30</v>
@@ -659,10 +659,10 @@
         <v>11</v>
       </c>
       <c r="C5" s="8">
-        <v>46054</v>
+        <v>46113</v>
       </c>
       <c r="D5" s="8">
-        <v>46234</v>
+        <v>46295</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>33</v>
@@ -676,10 +676,10 @@
         <v>13</v>
       </c>
       <c r="C6" s="8">
-        <v>46082</v>
+        <v>46143</v>
       </c>
       <c r="D6" s="8">
-        <v>46234</v>
+        <v>46295</v>
       </c>
       <c r="E6" s="9" t="s">
         <v>7</v>
@@ -693,10 +693,10 @@
         <v>15</v>
       </c>
       <c r="C7" s="8">
-        <v>46082</v>
+        <v>46143</v>
       </c>
       <c r="D7" s="8">
-        <v>46234</v>
+        <v>46295</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>7</v>
@@ -710,10 +710,10 @@
         <v>17</v>
       </c>
       <c r="C8" s="8">
-        <v>46082</v>
+        <v>46143</v>
       </c>
       <c r="D8" s="8">
-        <v>46173</v>
+        <v>46234</v>
       </c>
       <c r="E8" s="9" t="s">
         <v>18</v>
@@ -727,10 +727,10 @@
         <v>20</v>
       </c>
       <c r="C9" s="8">
-        <v>46082</v>
+        <v>46143</v>
       </c>
       <c r="D9" s="8">
-        <v>46112</v>
+        <v>46173</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>21</v>
@@ -744,10 +744,10 @@
         <v>23</v>
       </c>
       <c r="C10" s="8">
-        <v>46082</v>
+        <v>46143</v>
       </c>
       <c r="D10" s="8">
-        <v>46112</v>
+        <v>46173</v>
       </c>
       <c r="E10" s="9" t="s">
         <v>21</v>
@@ -761,10 +761,10 @@
         <v>24</v>
       </c>
       <c r="C11" s="8">
-        <v>46082</v>
+        <v>46143</v>
       </c>
       <c r="D11" s="8">
-        <v>46173</v>
+        <v>46234</v>
       </c>
       <c r="E11" s="9" t="s">
         <v>18</v>
@@ -778,10 +778,10 @@
         <v>25</v>
       </c>
       <c r="C12" s="8">
-        <v>46082</v>
+        <v>46143</v>
       </c>
       <c r="D12" s="8">
-        <v>46173</v>
+        <v>46234</v>
       </c>
       <c r="E12" s="9" t="s">
         <v>18</v>
@@ -795,10 +795,10 @@
         <v>27</v>
       </c>
       <c r="C13" s="8">
-        <v>46082</v>
+        <v>46143</v>
       </c>
       <c r="D13" s="8">
-        <v>46173</v>
+        <v>46234</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>18</v>
@@ -812,10 +812,10 @@
         <v>32</v>
       </c>
       <c r="C14" s="8">
-        <v>46082</v>
+        <v>46143</v>
       </c>
       <c r="D14" s="8">
-        <v>46112</v>
+        <v>46173</v>
       </c>
       <c r="E14" s="9" t="s">
         <v>21</v>
@@ -829,10 +829,10 @@
         <v>35</v>
       </c>
       <c r="C15" s="8">
-        <v>46082</v>
+        <v>46143</v>
       </c>
       <c r="D15" s="8">
-        <v>46112</v>
+        <v>46173</v>
       </c>
       <c r="E15" s="9" t="s">
         <v>21</v>

</xml_diff>

<commit_message>
chore: update capacity report script to june 2026
Update all hardcoded file paths, month constants, and report output directories in the capacity report script to use june 2026's planning folders, and remove the temporary excel lock file.
</commit_message>
<xml_diff>
--- a/FastReact Confg..xlsx
+++ b/FastReact Confg..xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\1. Work\1. Daily\Capacity Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19F83E07-8D07-4D4A-B6F6-9741F9826CB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0984D2CA-FEE9-4EC0-A258-C79349632CC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="810" yWindow="-120" windowWidth="19800" windowHeight="11760" xr2:uid="{9AFED8FC-535D-48D6-A46B-931961F691BE}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="33">
   <si>
     <t>Report Name</t>
   </si>
@@ -108,24 +108,6 @@
     <t>Reports- Planning- Buyer wise plan qty- Per_Day_Requirement (Unit)</t>
   </si>
   <si>
-    <t>Reports- Auto status- Buyer Wise Monthly print Req- Buyer Wise Monthly print Req.</t>
-  </si>
-  <si>
-    <t>Reports- Auto status- Buyer Wise Monthly Emb Req- Buyer Wise Monthly Emb Req.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BuyerWise Monthly Wash Req  </t>
-  </si>
-  <si>
-    <t>Reports- Auto status- Buyer Wise Monthly Wash Req- Buyer Wise Monthly Wash Req.</t>
-  </si>
-  <si>
-    <t>BuyerWise Monthly Emb Req</t>
-  </si>
-  <si>
-    <t>BuyerWise Monthly Print Req.</t>
-  </si>
-  <si>
     <t>Current Month + 5</t>
   </si>
   <si>
@@ -145,6 +127,12 @@
   </si>
   <si>
     <t>FastReact planning necessary report configurations</t>
+  </si>
+  <si>
+    <t>Unit wise Detail Plan</t>
+  </si>
+  <si>
+    <t>Reports-Production-UNITWISE DETAIL LINE PLAN-JFL Detail Plan</t>
   </si>
 </sst>
 </file>
@@ -580,7 +568,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{293FE00B-EC13-46E8-B78F-2F1EC25697CE}">
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.28515625" style="2" customWidth="1"/>
@@ -593,7 +581,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="29.25" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -625,10 +613,10 @@
         <v>6</v>
       </c>
       <c r="C3" s="8">
-        <v>46143</v>
+        <v>46235</v>
       </c>
       <c r="D3" s="8">
-        <v>46295</v>
+        <v>46387</v>
       </c>
       <c r="E3" s="9" t="s">
         <v>7</v>
@@ -642,13 +630,13 @@
         <v>9</v>
       </c>
       <c r="C4" s="8">
-        <v>46113</v>
+        <v>46204</v>
       </c>
       <c r="D4" s="8">
-        <v>46295</v>
+        <v>46387</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="45" x14ac:dyDescent="0.25">
@@ -659,13 +647,13 @@
         <v>11</v>
       </c>
       <c r="C5" s="8">
-        <v>46113</v>
+        <v>46204</v>
       </c>
       <c r="D5" s="8">
-        <v>46295</v>
+        <v>46387</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="45" x14ac:dyDescent="0.25">
@@ -676,10 +664,10 @@
         <v>13</v>
       </c>
       <c r="C6" s="8">
-        <v>46143</v>
+        <v>46235</v>
       </c>
       <c r="D6" s="8">
-        <v>46295</v>
+        <v>46387</v>
       </c>
       <c r="E6" s="9" t="s">
         <v>7</v>
@@ -693,10 +681,10 @@
         <v>15</v>
       </c>
       <c r="C7" s="8">
-        <v>46143</v>
+        <v>46235</v>
       </c>
       <c r="D7" s="8">
-        <v>46295</v>
+        <v>46387</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>7</v>
@@ -710,10 +698,10 @@
         <v>17</v>
       </c>
       <c r="C8" s="8">
-        <v>46143</v>
+        <v>46235</v>
       </c>
       <c r="D8" s="8">
-        <v>46234</v>
+        <v>46326</v>
       </c>
       <c r="E8" s="9" t="s">
         <v>18</v>
@@ -727,10 +715,10 @@
         <v>20</v>
       </c>
       <c r="C9" s="8">
-        <v>46143</v>
+        <v>46235</v>
       </c>
       <c r="D9" s="8">
-        <v>46173</v>
+        <v>46265</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>21</v>
@@ -744,97 +732,63 @@
         <v>23</v>
       </c>
       <c r="C10" s="8">
-        <v>46143</v>
+        <v>46235</v>
       </c>
       <c r="D10" s="8">
-        <v>46173</v>
+        <v>46265</v>
       </c>
       <c r="E10" s="9" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C11" s="8">
-        <v>46143</v>
+        <v>46235</v>
       </c>
       <c r="D11" s="8">
-        <v>46234</v>
+        <v>46265</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>28</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C12" s="8">
-        <v>46143</v>
+        <v>46235</v>
       </c>
       <c r="D12" s="8">
-        <v>46234</v>
+        <v>46265</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C13" s="8">
-        <v>46143</v>
+        <v>46235</v>
       </c>
       <c r="D13" s="8">
-        <v>46234</v>
+        <v>46265</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="C14" s="8">
-        <v>46143</v>
-      </c>
-      <c r="D14" s="8">
-        <v>46173</v>
-      </c>
-      <c r="E14" s="9" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A15" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="C15" s="8">
-        <v>46143</v>
-      </c>
-      <c r="D15" s="8">
-        <v>46173</v>
-      </c>
-      <c r="E15" s="9" t="s">
         <v>21</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(capacity_report): update setup for aug 2026
modify input/output file paths and month constants to target august 2026 directories, and refresh associated template and config excel files
</commit_message>
<xml_diff>
--- a/FastReact Confg..xlsx
+++ b/FastReact Confg..xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\1. Work\1. Daily\Capacity Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0984D2CA-FEE9-4EC0-A258-C79349632CC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2E0DC10-BE70-4FB1-9851-25C8C0EC716D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="810" yWindow="-120" windowWidth="19800" windowHeight="11760" xr2:uid="{9AFED8FC-535D-48D6-A46B-931961F691BE}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="35">
   <si>
     <t>Report Name</t>
   </si>
@@ -133,6 +133,12 @@
   </si>
   <si>
     <t>Reports-Production-UNITWISE DETAIL LINE PLAN-JFL Detail Plan</t>
+  </si>
+  <si>
+    <t>Blank Days Per Month</t>
+  </si>
+  <si>
+    <t>JFL Monthly</t>
   </si>
 </sst>
 </file>
@@ -568,7 +574,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{293FE00B-EC13-46E8-B78F-2F1EC25697CE}">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.28515625" style="2" customWidth="1"/>
@@ -613,10 +619,10 @@
         <v>6</v>
       </c>
       <c r="C3" s="8">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="D3" s="8">
-        <v>46387</v>
+        <v>46418</v>
       </c>
       <c r="E3" s="9" t="s">
         <v>7</v>
@@ -630,10 +636,10 @@
         <v>9</v>
       </c>
       <c r="C4" s="8">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="D4" s="8">
-        <v>46387</v>
+        <v>46418</v>
       </c>
       <c r="E4" s="9" t="s">
         <v>24</v>
@@ -647,10 +653,10 @@
         <v>11</v>
       </c>
       <c r="C5" s="8">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="D5" s="8">
-        <v>46387</v>
+        <v>46418</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>27</v>
@@ -664,10 +670,10 @@
         <v>13</v>
       </c>
       <c r="C6" s="8">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="D6" s="8">
-        <v>46387</v>
+        <v>46418</v>
       </c>
       <c r="E6" s="9" t="s">
         <v>7</v>
@@ -681,10 +687,10 @@
         <v>15</v>
       </c>
       <c r="C7" s="8">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="D7" s="8">
-        <v>46387</v>
+        <v>46418</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>7</v>
@@ -698,10 +704,10 @@
         <v>17</v>
       </c>
       <c r="C8" s="8">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="D8" s="8">
-        <v>46326</v>
+        <v>46356</v>
       </c>
       <c r="E8" s="9" t="s">
         <v>18</v>
@@ -715,10 +721,10 @@
         <v>20</v>
       </c>
       <c r="C9" s="8">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="D9" s="8">
-        <v>46265</v>
+        <v>46295</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>21</v>
@@ -732,10 +738,10 @@
         <v>23</v>
       </c>
       <c r="C10" s="8">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="D10" s="8">
-        <v>46265</v>
+        <v>46295</v>
       </c>
       <c r="E10" s="9" t="s">
         <v>21</v>
@@ -749,10 +755,10 @@
         <v>26</v>
       </c>
       <c r="C11" s="8">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="D11" s="8">
-        <v>46265</v>
+        <v>46295</v>
       </c>
       <c r="E11" s="9" t="s">
         <v>21</v>
@@ -766,10 +772,10 @@
         <v>29</v>
       </c>
       <c r="C12" s="8">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="D12" s="8">
-        <v>46265</v>
+        <v>46295</v>
       </c>
       <c r="E12" s="9" t="s">
         <v>21</v>
@@ -783,12 +789,29 @@
         <v>32</v>
       </c>
       <c r="C13" s="8">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="D13" s="8">
-        <v>46265</v>
+        <v>46295</v>
       </c>
       <c r="E13" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14" s="8">
+        <v>46266</v>
+      </c>
+      <c r="D14" s="8">
+        <v>46295</v>
+      </c>
+      <c r="E14" s="9" t="s">
         <v>21</v>
       </c>
     </row>

</xml_diff>